<commit_message>
Final commit before submission
</commit_message>
<xml_diff>
--- a/backend/financial_report.xlsx
+++ b/backend/financial_report.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -460,6 +460,52 @@
       <c r="E2" t="inlineStr">
         <is>
           <t>2026-06-24 23:07:17.958224</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B3" t="n">
+        <v>500000</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Salary</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>First stipend</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-06-25 21:27:45.192764</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B4" t="n">
+        <v>20000</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Stipend</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Nelfund</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-06-25 22:02:48.670087</t>
         </is>
       </c>
     </row>
@@ -474,7 +520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -524,6 +570,29 @@
       <c r="E2" t="inlineStr">
         <is>
           <t>2026-06-24 23:21:17.984590</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="n">
+        <v>100000</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Body accessories </t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Birthday dress</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-06-25 21:29:47.039555</t>
         </is>
       </c>
     </row>

</xml_diff>